<commit_message>
add posting date to stock NCR template
</commit_message>
<xml_diff>
--- a/public/template-stok-ncr-grade-c.xlsx
+++ b/public/template-stok-ncr-grade-c.xlsx
@@ -1,55 +1,110 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Stok Grade C" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Stok Grade C" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+  <si>
+    <t>SLOC</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>MATERIAL NUMBER</t>
+  </si>
+  <si>
+    <t>DIAM "</t>
+  </si>
+  <si>
+    <t>LENGTH SIDE</t>
+  </si>
+  <si>
+    <t>WIDTH SIDE</t>
+  </si>
+  <si>
+    <t>DIAM MM</t>
+  </si>
+  <si>
+    <t>TEBAL</t>
+  </si>
+  <si>
+    <t>PANJANG</t>
+  </si>
+  <si>
+    <t>Unrestricted Pcs</t>
+  </si>
+  <si>
+    <t>Unrestricted Kg</t>
+  </si>
+  <si>
+    <t>BATCH</t>
+  </si>
+  <si>
+    <t>NOMOR SO</t>
+  </si>
+  <si>
+    <t>ITEM SO</t>
+  </si>
+  <si>
+    <t>Requested deliv.date</t>
+  </si>
+  <si>
+    <t>CUST.REMARK</t>
+  </si>
+  <si>
+    <t>Forecats Cust.</t>
+  </si>
+  <si>
+    <t>PASM</t>
+  </si>
+  <si>
+    <t>PASG</t>
+  </si>
+  <si>
+    <t>BLOK STOK BOm</t>
+  </si>
+  <si>
+    <t>Post.Date</t>
+  </si>
+  <si>
+    <t>XX</t>
+  </si>
+  <si>
+    <t>Gudang</t>
+  </si>
+  <si>
+    <t>Panjang Pipa</t>
+  </si>
+  <si>
+    <t>ST/LT</t>
+  </si>
+  <si>
+    <t>Grade</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="9">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="58" formatCode="m/d/yy"/>
-    <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;Rp&quot;* #,##0.00_-;\-&quot;Rp&quot;* #,##0.00_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="180" formatCode="0.000"/>
-    <numFmt numFmtId="181" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="182" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -72,14 +127,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -404,93 +470,95 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Z1"/>
+  <sheetFormatPr customHeight="1"/>
   <cols>
-    <col min="12" max="12" customWidth="1" width="13.4285714285714"/>
+    <col min="12" max="12" width="13.4285714285714" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="38.25" customHeight="1">
-      <c r="A1" t="str">
-        <v>SLOC</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Customer</v>
-      </c>
-      <c r="C1" t="str">
-        <v>MATERIAL NUMBER</v>
-      </c>
-      <c r="D1" t="str">
-        <v>DIAM "</v>
-      </c>
-      <c r="E1" t="str">
-        <v>LENGTH SIDE</v>
-      </c>
-      <c r="F1" t="str">
-        <v>WIDTH SIDE</v>
-      </c>
-      <c r="G1" t="str">
-        <v>DIAM MM</v>
-      </c>
-      <c r="H1" t="str">
-        <v>TEBAL</v>
-      </c>
-      <c r="I1" t="str">
-        <v>PANJANG</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Unrestricted Pcs</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Unrestricted Kg</v>
-      </c>
-      <c r="L1" t="str">
-        <v>BATCH</v>
-      </c>
-      <c r="M1" t="str">
-        <v>NOMOR SO</v>
-      </c>
-      <c r="N1" t="str">
-        <v>ITEM SO</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Requested deliv.date</v>
-      </c>
-      <c r="P1" t="str">
-        <v>CUST.REMARK</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Forecats Cust.</v>
-      </c>
-      <c r="R1" t="str">
-        <v>PASM</v>
-      </c>
-      <c r="S1" t="str">
-        <v>PASG</v>
-      </c>
-      <c r="T1" t="str">
-        <v>BLOK STOK BOm</v>
-      </c>
-      <c r="U1" t="str">
-        <v>XX</v>
-      </c>
-      <c r="V1" t="str">
-        <v>Gudang</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Panjang Pipa</v>
-      </c>
-      <c r="X1" t="str">
-        <v>ST/LT</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>Grade</v>
+    <row r="1" ht="38.25" customHeight="1" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y2"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>